<commit_message>
[ OK ] Funciona la base de datos de DuckDB
</commit_message>
<xml_diff>
--- a/models/plantilla_consolidado_he.xlsx
+++ b/models/plantilla_consolidado_he.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Revisar_primero" sheetId="1" state="visible" r:id="rId3"/>
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Cuadrilla</t>
   </si>
   <si>
-    <t xml:space="preserve">Responsable</t>
+    <t xml:space="preserve">Colaboradores</t>
   </si>
   <si>
     <t xml:space="preserve">Dia</t>
@@ -1342,13 +1342,13 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="31.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="39.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="23.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="18" width="14.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="19" width="16.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="20" width="14.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="20" width="13.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="21" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="22" width="170.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="22" width="114.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="10.14"/>

</xml_diff>

<commit_message>
[ Test ] initials refactor and group. Also, New Free Day on plantilla
</commit_message>
<xml_diff>
--- a/models/plantilla_consolidado_he.xlsx
+++ b/models/plantilla_consolidado_he.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Revisar_primero" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="78">
   <si>
     <t xml:space="preserve">Aplica</t>
   </si>
@@ -170,13 +170,16 @@
     <t xml:space="preserve"> lunch</t>
   </si>
   <si>
+    <t xml:space="preserve">“Dia Festivo: Decreto 431”</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zamora Z1 (Cuadrilla. Nro. 6)</t>
   </si>
   <si>
     <t xml:space="preserve">“Dia Festivo: Cantonizacion”</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ?</t>
   </si>
   <si>
     <t xml:space="preserve">Zamora Z1 (Cuadrilla. AP Nro. 4)</t>
@@ -1089,31 +1092,31 @@
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>46300</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="E16" s="2"/>
       <c r="J16" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>46139</v>
@@ -1128,7 +1131,7 @@
         <v>46300</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>46140</v>
@@ -1143,7 +1146,7 @@
         <v>46300</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>46141</v>
@@ -1155,10 +1158,10 @@
         <v>54</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>46031</v>
+        <v>46300</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>46160</v>
@@ -1170,10 +1173,10 @@
         <v>55</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>46080</v>
+        <v>46031</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>46161</v>
@@ -1188,7 +1191,7 @@
         <v>46080</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>46162</v>
@@ -1203,7 +1206,7 @@
         <v>46080</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>46163</v>
@@ -1215,10 +1218,10 @@
         <v>58</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46319</v>
+        <v>46080</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>46174</v>
@@ -1230,10 +1233,10 @@
         <v>59</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>46353</v>
+        <v>46319</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -1243,10 +1246,10 @@
         <v>60</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>46065</v>
+        <v>46353</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -1259,7 +1262,7 @@
         <v>46065</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1269,10 +1272,10 @@
         <v>62</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>46251</v>
+        <v>46065</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
@@ -1285,12 +1288,21 @@
         <v>46251</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
@@ -1359,46 +1371,46 @@
   <sheetData>
     <row r="1" s="23" customFormat="true" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D1" s="24" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K1" s="23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L1" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M1" s="23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N1" s="23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
[ OK ] Sinronizcion con XPS Delta
</commit_message>
<xml_diff>
--- a/models/plantilla_consolidado_he.xlsx
+++ b/models/plantilla_consolidado_he.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Revisar_primero" sheetId="1" state="visible" r:id="rId3"/>
@@ -527,8 +527,8 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -548,15 +548,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1360,12 +1360,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="20" width="14.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="20" width="13.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="21" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="22" width="114.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="55.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="22.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="17" width="114.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="22" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="22" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="22" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="22" width="55.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="22" width="22.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="13.42"/>
   </cols>
   <sheetData>

</xml_diff>